<commit_message>
Copilot cleaned the methodology notebook, improving latex and overall placement without changing the methodology
</commit_message>
<xml_diff>
--- a/INPUTS/Proyeccion_2026.xlsx
+++ b/INPUTS/Proyeccion_2026.xlsx
@@ -319,6 +319,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -328,7 +329,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -689,18 +689,18 @@
       <c r="F2" s="7">
         <v>90255206894.380005</v>
       </c>
-      <c r="I2" s="9" t="s">
+      <c r="I2" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="J2" s="9"/>
-      <c r="L2" s="10" t="s">
+      <c r="J2" s="10"/>
+      <c r="L2" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="M2" s="10"/>
-      <c r="N2" s="10"/>
-      <c r="O2" s="10"/>
-      <c r="P2" s="10"/>
-      <c r="Q2" s="10"/>
+      <c r="M2" s="11"/>
+      <c r="N2" s="11"/>
+      <c r="O2" s="11"/>
+      <c r="P2" s="11"/>
+      <c r="Q2" s="11"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -728,14 +728,14 @@
         <f>G30</f>
         <v>9.6886196108379785E-2</v>
       </c>
-      <c r="L3" s="11" t="s">
+      <c r="L3" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="M3" s="11"/>
-      <c r="N3" s="11"/>
-      <c r="O3" s="11"/>
-      <c r="P3" s="11"/>
-      <c r="Q3" s="11"/>
+      <c r="M3" s="12"/>
+      <c r="N3" s="12"/>
+      <c r="O3" s="12"/>
+      <c r="P3" s="12"/>
+      <c r="Q3" s="12"/>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
@@ -768,12 +768,12 @@
         <f>(F2/B2)^(1/5)-1</f>
         <v>7.6465659507858774E-2</v>
       </c>
-      <c r="L4" s="11"/>
-      <c r="M4" s="11"/>
-      <c r="N4" s="11"/>
-      <c r="O4" s="11"/>
-      <c r="P4" s="11"/>
-      <c r="Q4" s="11"/>
+      <c r="L4" s="12"/>
+      <c r="M4" s="12"/>
+      <c r="N4" s="12"/>
+      <c r="O4" s="12"/>
+      <c r="P4" s="12"/>
+      <c r="Q4" s="12"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
@@ -801,12 +801,12 @@
         <f>AVERAGE(E30:F30)</f>
         <v>6.787330490688781E-2</v>
       </c>
-      <c r="L5" s="11"/>
-      <c r="M5" s="11"/>
-      <c r="N5" s="11"/>
-      <c r="O5" s="11"/>
-      <c r="P5" s="11"/>
-      <c r="Q5" s="11"/>
+      <c r="L5" s="12"/>
+      <c r="M5" s="12"/>
+      <c r="N5" s="12"/>
+      <c r="O5" s="12"/>
+      <c r="P5" s="12"/>
+      <c r="Q5" s="12"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
@@ -827,12 +827,12 @@
       <c r="F6" s="7">
         <v>85048136203.669998</v>
       </c>
-      <c r="L6" s="11"/>
-      <c r="M6" s="11"/>
-      <c r="N6" s="11"/>
-      <c r="O6" s="11"/>
-      <c r="P6" s="11"/>
-      <c r="Q6" s="11"/>
+      <c r="L6" s="12"/>
+      <c r="M6" s="12"/>
+      <c r="N6" s="12"/>
+      <c r="O6" s="12"/>
+      <c r="P6" s="12"/>
+      <c r="Q6" s="12"/>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
@@ -853,16 +853,16 @@
       <c r="F7" s="7">
         <v>13517235117.35</v>
       </c>
-      <c r="I7" s="9" t="s">
+      <c r="I7" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="J7" s="9"/>
-      <c r="L7" s="11"/>
-      <c r="M7" s="11"/>
-      <c r="N7" s="11"/>
-      <c r="O7" s="11"/>
-      <c r="P7" s="11"/>
-      <c r="Q7" s="11"/>
+      <c r="J7" s="10"/>
+      <c r="L7" s="12"/>
+      <c r="M7" s="12"/>
+      <c r="N7" s="12"/>
+      <c r="O7" s="12"/>
+      <c r="P7" s="12"/>
+      <c r="Q7" s="12"/>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
@@ -917,14 +917,14 @@
         <f>SUM(B3:F3)/SUM(B2:F2)</f>
         <v>3.7143863998180496E-2</v>
       </c>
-      <c r="L9" s="11" t="s">
+      <c r="L9" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="M9" s="11"/>
-      <c r="N9" s="11"/>
-      <c r="O9" s="11"/>
-      <c r="P9" s="11"/>
-      <c r="Q9" s="11"/>
+      <c r="M9" s="12"/>
+      <c r="N9" s="12"/>
+      <c r="O9" s="12"/>
+      <c r="P9" s="12"/>
+      <c r="Q9" s="12"/>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
@@ -945,12 +945,12 @@
       <c r="F10" s="7">
         <v>12583277072.24</v>
       </c>
-      <c r="L10" s="11"/>
-      <c r="M10" s="11"/>
-      <c r="N10" s="11"/>
-      <c r="O10" s="11"/>
-      <c r="P10" s="11"/>
-      <c r="Q10" s="11"/>
+      <c r="L10" s="12"/>
+      <c r="M10" s="12"/>
+      <c r="N10" s="12"/>
+      <c r="O10" s="12"/>
+      <c r="P10" s="12"/>
+      <c r="Q10" s="12"/>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
@@ -971,16 +971,16 @@
       <c r="F11" s="7">
         <v>129993857280.42999</v>
       </c>
-      <c r="I11" s="9" t="s">
+      <c r="I11" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="J11" s="9"/>
-      <c r="L11" s="11"/>
-      <c r="M11" s="11"/>
-      <c r="N11" s="11"/>
-      <c r="O11" s="11"/>
-      <c r="P11" s="11"/>
-      <c r="Q11" s="11"/>
+      <c r="J11" s="10"/>
+      <c r="L11" s="12"/>
+      <c r="M11" s="12"/>
+      <c r="N11" s="12"/>
+      <c r="O11" s="12"/>
+      <c r="P11" s="12"/>
+      <c r="Q11" s="12"/>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B12" s="7"/>
@@ -995,12 +995,12 @@
         <f>G33</f>
         <v>0.94566475101261138</v>
       </c>
-      <c r="L12" s="11"/>
-      <c r="M12" s="11"/>
-      <c r="N12" s="11"/>
-      <c r="O12" s="11"/>
-      <c r="P12" s="11"/>
-      <c r="Q12" s="11"/>
+      <c r="L12" s="12"/>
+      <c r="M12" s="12"/>
+      <c r="N12" s="12"/>
+      <c r="O12" s="12"/>
+      <c r="P12" s="12"/>
+      <c r="Q12" s="12"/>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B13" s="7"/>
@@ -1015,12 +1015,12 @@
         <f>SUM(B6:F6)/SUM(B4:F4)</f>
         <v>0.94680421611380128</v>
       </c>
-      <c r="L13" s="11"/>
-      <c r="M13" s="11"/>
-      <c r="N13" s="11"/>
-      <c r="O13" s="11"/>
-      <c r="P13" s="11"/>
-      <c r="Q13" s="11"/>
+      <c r="L13" s="12"/>
+      <c r="M13" s="12"/>
+      <c r="N13" s="12"/>
+      <c r="O13" s="12"/>
+      <c r="P13" s="12"/>
+      <c r="Q13" s="12"/>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B14" s="7"/>
@@ -1051,10 +1051,10 @@
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
-      <c r="I16" s="9" t="s">
+      <c r="I16" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="J16" s="9"/>
+      <c r="J16" s="10"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
@@ -1110,7 +1110,7 @@
       <c r="I18" t="s">
         <v>42</v>
       </c>
-      <c r="J18" s="12">
+      <c r="J18" s="9">
         <f>SUM(B7:F7)/SUM(B2:F2)</f>
         <v>0.1514241742958887</v>
       </c>
@@ -1158,10 +1158,10 @@
         <f t="shared" si="1"/>
         <v>0.12763969780383055</v>
       </c>
-      <c r="I20" s="9" t="s">
+      <c r="I20" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="J20" s="9"/>
+      <c r="J20" s="10"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
@@ -1217,7 +1217,7 @@
       <c r="I22" t="s">
         <v>54</v>
       </c>
-      <c r="J22" s="12">
+      <c r="J22" s="9">
         <f>AVERAGE(E40:F40)</f>
         <v>0.70999392967041675</v>
       </c>
@@ -1293,10 +1293,10 @@
       <c r="F25" s="3">
         <v>12583277072.24</v>
       </c>
-      <c r="I25" s="9" t="s">
+      <c r="I25" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="J25" s="9"/>
+      <c r="J25" s="10"/>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
@@ -1507,23 +1507,23 @@
       <c r="A34" t="s">
         <v>47</v>
       </c>
-      <c r="B34" s="12">
+      <c r="B34" s="9">
         <f>B17/B2</f>
         <v>0.13970566410904758</v>
       </c>
-      <c r="C34" s="12">
+      <c r="C34" s="9">
         <f t="shared" ref="C34:F34" si="7">C17/C2</f>
         <v>0.14037811670425721</v>
       </c>
-      <c r="D34" s="12">
+      <c r="D34" s="9">
         <f t="shared" si="7"/>
         <v>0.17237525596371353</v>
       </c>
-      <c r="E34" s="12">
+      <c r="E34" s="9">
         <f t="shared" si="7"/>
         <v>0.15133840575222382</v>
       </c>
-      <c r="F34" s="12">
+      <c r="F34" s="9">
         <f t="shared" si="7"/>
         <v>0.14976681769915359</v>
       </c>
@@ -1626,15 +1626,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="L2:Q2"/>
+    <mergeCell ref="L3:Q7"/>
+    <mergeCell ref="L9:Q13"/>
+    <mergeCell ref="I11:J11"/>
     <mergeCell ref="I20:J20"/>
     <mergeCell ref="I16:J16"/>
     <mergeCell ref="I25:J25"/>
     <mergeCell ref="I2:J2"/>
     <mergeCell ref="I7:J7"/>
-    <mergeCell ref="L2:Q2"/>
-    <mergeCell ref="L3:Q7"/>
-    <mergeCell ref="L9:Q13"/>
-    <mergeCell ref="I11:J11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>